<commit_message>
Update ES2N-Requisitos Funcionais v4.0.xlsx
</commit_message>
<xml_diff>
--- a/Requisitos Funcionais/ES2N-Requisitos Funcionais v4.0.xlsx
+++ b/Requisitos Funcionais/ES2N-Requisitos Funcionais v4.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://toyotabrasil-my.sharepoint.com/personal/aaloliveira_toyota_com_br/Documents/Documentos/GitHub/deploynasexta/Requisitos Funcionais/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_26AEB4EC332602B7D99C5FBD30863A8819128564" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{808E047F-E561-43C9-B7DC-2F92F1C33063}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_26AEB4EC332602B7D99C5FBD30863A8819128564" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DEC2327-C7AC-4D2E-A69F-25DFFD25E375}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
   <si>
     <t xml:space="preserve">LISTA DE REQUISITOS FUNCIONAIS </t>
   </si>
@@ -80,9 +80,6 @@
     <t>Alta</t>
   </si>
   <si>
-    <t>Depende do requisito RF02.</t>
-  </si>
-  <si>
     <t>RF02</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
     <t>O sistema deve permitir que o usuário interno encerre sua sessão de uso de forma segura.</t>
   </si>
   <si>
-    <t>Encerra a sessão iniciada pelo requisito RF02.</t>
-  </si>
-  <si>
     <t>RF04</t>
   </si>
   <si>
@@ -119,9 +113,6 @@
     <t>Média</t>
   </si>
   <si>
-    <t>Pode ser executado a partir do requisito RF02.</t>
-  </si>
-  <si>
     <t>RF05</t>
   </si>
   <si>
@@ -134,9 +125,6 @@
     <t>Administrador e Colaborador</t>
   </si>
   <si>
-    <t>Pode apoiar a execução do requisito RF06.</t>
-  </si>
-  <si>
     <t>RF06</t>
   </si>
   <si>
@@ -146,9 +134,6 @@
     <t>O sistema deve permitir cadastrar, alterar, consultar e cancelar solicitações de retirada de doações, registrando data, período do dia, endereço, item a ser doado e responsável pelo atendimento.</t>
   </si>
   <si>
-    <t>Pode executar o requisito RF07.</t>
-  </si>
-  <si>
     <t>RF07</t>
   </si>
   <si>
@@ -158,9 +143,6 @@
     <t>O sistema deve permitir registrar entradas e saídas de itens no estoque a partir do recebimento de doações e da distribuição de itens, mantendo o saldo atualizado.</t>
   </si>
   <si>
-    <t>Atualiza informações utilizadas nos requisitos RF08, RF09 e RF14.</t>
-  </si>
-  <si>
     <t>RF08</t>
   </si>
   <si>
@@ -170,9 +152,6 @@
     <t>O sistema deve permitir consultar o estoque com pesquisa e filtragem por nome do item, categoria, validade e disponibilidade.</t>
   </si>
   <si>
-    <t>Pode apoiar a execução dos requisitos RF06, RF07, RF09 e RF14.</t>
-  </si>
-  <si>
     <t>RF09</t>
   </si>
   <si>
@@ -182,18 +161,12 @@
     <t>O sistema deve permitir gerar relatórios de doações recebidas, movimentação de estoque e itens próximos do vencimento, com filtro por período.</t>
   </si>
   <si>
-    <t>Utiliza dados dos requisitos RF05 a RF08 e RF10 a RF13.</t>
-  </si>
-  <si>
     <t>RF10</t>
   </si>
   <si>
     <t>Gerenciar categorias</t>
   </si>
   <si>
-    <t>Pode ser executado antes dos requisitos RF11 e RF12.</t>
-  </si>
-  <si>
     <t>RF11</t>
   </si>
   <si>
@@ -218,9 +191,6 @@
     <t>Sistema</t>
   </si>
   <si>
-    <t>Pode apoiar a execução dos requisitos RF08, RF09 e RF14.</t>
-  </si>
-  <si>
     <t>RF14</t>
   </si>
   <si>
@@ -228,9 +198,6 @@
   </si>
   <si>
     <t>O sistema deve apresentar um painel com indicadores de doações recebidas, movimentação de estoque, itens próximos do vencimento e doadores ativos.</t>
-  </si>
-  <si>
-    <t>Utiliza dados consolidados dos requisitos RF05 a RF13.</t>
   </si>
   <si>
     <t>*** Observação: o termo 'Gerenciar' é utilizado quando o requisito contempla operações de consulta, cadastro, alteração e inativação/exclusão lógica, conforme orientação da professora.</t>
@@ -759,7 +726,7 @@
     </row>
     <row r="4" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A4" s="1" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="B4" s="1"/>
     </row>
@@ -809,240 +776,220 @@
       <c r="E10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>15</v>
-      </c>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
       <c r="A12" s="8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="D12" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>19</v>
-      </c>
       <c r="E12" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>78</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="47" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>22</v>
-      </c>
       <c r="D13" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>23</v>
-      </c>
+      <c r="F13" s="8"/>
     </row>
     <row r="14" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B14" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>28</v>
-      </c>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:6" ht="94" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="8" t="s">
-        <v>33</v>
-      </c>
+      <c r="F15" s="8"/>
     </row>
     <row r="16" spans="1:6" ht="94" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="F16" s="8"/>
     </row>
     <row r="17" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>41</v>
-      </c>
+      <c r="F17" s="8"/>
     </row>
     <row r="18" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>45</v>
-      </c>
+      <c r="F18" s="8"/>
     </row>
     <row r="19" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>65</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="F19" s="8"/>
     </row>
     <row r="20" spans="1:6" ht="70.5" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D20" s="8" t="s">
         <v>13</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>49</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="F20" s="8"/>
     </row>
     <row r="21" spans="1:6" ht="94" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F21" s="8" t="s">
-        <v>52</v>
-      </c>
+      <c r="F21" s="8"/>
     </row>
     <row r="22" spans="1:6" ht="94" x14ac:dyDescent="0.35">
       <c r="A22" s="8" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
       <c r="D22" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>14</v>
@@ -1051,67 +998,61 @@
     </row>
     <row r="23" spans="1:6" ht="117.5" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F23" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="F23" s="8"/>
     </row>
     <row r="24" spans="1:6" ht="94" x14ac:dyDescent="0.35">
       <c r="A24" s="8" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F24" s="8" t="s">
-        <v>37</v>
-      </c>
+      <c r="F24" s="8"/>
     </row>
     <row r="25" spans="1:6" ht="72" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="8" t="s">
-        <v>61</v>
-      </c>
+      <c r="F25" s="8"/>
     </row>
     <row r="27" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="9" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="10"/>

</xml_diff>